<commit_message>
Fix live puzzle rsz-009 in place and guard against stale saved state
rsz-009 (2026-10-01) had factual errors: "Indián" is not a palindrome and
"Nadrág" does not naturally have a "lába". Same id and date, new groups:
Fűszerek / SZÉL + ___ / Oda-vissza ugyanaz / ___ + LÁB.

- xlsx_to_js.py: one-off `--javitas <id>` flag lets the workbook override
  a single live puzzle for that run (date may not change). Without it the
  live-puzzle lock works as before; CI never passes it.
- jatek.js: on load, if a saved state for the puzzle references words not
  in it, an in-progress game resets to a fresh board; a finished game keeps
  its result. Stats/streak untouched; rokonszavak-v1 format unchanged.
- build.py: asset version hash ignores line endings so a Windows build
  matches the GitHub build.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feladvanyok.xlsx
+++ b/feladvanyok.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a3b2d023d0b90a2/Dokumentumok/Rokonszavak/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a3b2d023d0b90a2/Dokumentumok/GitHub/rokonszavak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_4BC928A0A355CC1831E4553E7CBF07CDD619E1D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88C53B5C-FD94-4B47-B9C2-AD49D1DE2B38}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_4BC928A0A355CC1831E4553E7CBF07CDD619E1D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{628C337C-280F-4B15-A767-E1BC83D40D2F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Útmutató" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Segéd" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="Játék" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="468">
   <si>
     <t>Rokonszavak – feladványbank és gyakorlólap</t>
   </si>
@@ -1431,6 +1431,18 @@
   </si>
   <si>
     <t>Öv</t>
+  </si>
+  <si>
+    <t>Oda-vissza ugyanaz</t>
+  </si>
+  <si>
+    <t>Sas</t>
+  </si>
+  <si>
+    <t>___ + LÁB</t>
+  </si>
+  <si>
+    <t>Kamat</t>
   </si>
 </sst>
 </file>
@@ -1449,21 +1461,21 @@
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1484,25 +1496,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.39997558519241921"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1544,6 +1550,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1551,9 +1560,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1639,6 +1645,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2821,13 +2831,13 @@
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>187</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>189</v>
@@ -2849,16 +2859,16 @@
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>193</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="J31" s="5"/>
     </row>
@@ -2873,20 +2883,20 @@
         <v>3</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>195</v>
+        <v>464</v>
       </c>
       <c r="E32" s="5"/>
       <c r="F32" s="5" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>199</v>
+        <v>465</v>
       </c>
       <c r="J32" s="5"/>
     </row>
@@ -2901,20 +2911,20 @@
         <v>4</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>200</v>
+        <v>466</v>
       </c>
       <c r="E33" s="5"/>
       <c r="F33" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>203</v>
+        <v>467</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>204</v>
+        <v>141</v>
       </c>
       <c r="J33" s="5"/>
     </row>
@@ -8213,7 +8223,11 @@
         <v>457</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>50</v>
+        <v>183</v>
+      </c>
+      <c r="C2" t="str">
+        <f>VLOOKUP(B2,Feladványok!A:B,2,FALSE)</f>
+        <v>2026-10-01</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -8222,75 +8236,75 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="str">
+      <c r="A6" s="10" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+1-1)</f>
-        <v>Ikrek</v>
+        <v>Indián</v>
       </c>
       <c r="B6" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+2-1)</f>
-        <v>Puli</v>
-      </c>
-      <c r="C6" s="9" t="str">
+        <v>Szék</v>
+      </c>
+      <c r="C6" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+3-1)</f>
-        <v>Csat</v>
-      </c>
-      <c r="D6" s="10" t="str">
+        <v>Kapor</v>
+      </c>
+      <c r="D6" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+4-1)</f>
-        <v>Rest</v>
+        <v>Csend</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="str">
+      <c r="A7" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+5-1)</f>
-        <v>Pumi</v>
-      </c>
-      <c r="B7" s="8" t="str">
+        <v>Görög</v>
+      </c>
+      <c r="B7" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+6-1)</f>
-        <v>Bika</v>
-      </c>
-      <c r="C7" s="8" t="str">
+        <v>Kerek</v>
+      </c>
+      <c r="C7" s="10" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+7-1)</f>
-        <v>Rák</v>
-      </c>
-      <c r="D7" s="9" t="str">
+        <v>Bors</v>
+      </c>
+      <c r="D7" s="10" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+8-1)</f>
-        <v>Cipő</v>
+        <v>Vihar</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="str">
+      <c r="A8" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+9-1)</f>
-        <v>Bélés</v>
-      </c>
-      <c r="B8" s="10" t="str">
+        <v>Pap</v>
+      </c>
+      <c r="B8" s="9" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+10-1)</f>
-        <v>Volna</v>
-      </c>
-      <c r="C8" s="9" t="str">
+        <v>Kömény</v>
+      </c>
+      <c r="C8" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+11-1)</f>
-        <v>Mérleg</v>
-      </c>
-      <c r="D8" s="7" t="str">
+        <v>Gomba</v>
+      </c>
+      <c r="D8" s="9" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+12-1)</f>
-        <v>Vizsla</v>
+        <v>Kakas</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="str">
+      <c r="A9" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+13-1)</f>
-        <v>Fehér</v>
-      </c>
-      <c r="B9" s="8" t="str">
+        <v>Babér</v>
+      </c>
+      <c r="B9" s="9" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+14-1)</f>
-        <v>Kos</v>
+        <v>Malom</v>
       </c>
       <c r="C9" s="9" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+15-1)</f>
-        <v>Harang</v>
-      </c>
-      <c r="D9" s="7" t="str">
+        <v>Asztal</v>
+      </c>
+      <c r="D9" s="10" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+16-1)</f>
-        <v>Kuvasz</v>
+        <v>Nadrág</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -8321,23 +8335,23 @@
       </c>
       <c r="B23" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Csillagjegyek</v>
+        <v>Fűszerek</v>
       </c>
       <c r="C23" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Rák</v>
+        <v>Kömény</v>
       </c>
       <c r="D23" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Kos</v>
+        <v>Bors</v>
       </c>
       <c r="E23" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Bika</v>
+        <v>Kapor</v>
       </c>
       <c r="F23" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Ikrek</v>
+        <v>Babér</v>
       </c>
       <c r="G23" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1))</f>
@@ -8350,23 +8364,23 @@
       </c>
       <c r="B24" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Magyar kutyafajták</v>
+        <v>SZÉL + ___</v>
       </c>
       <c r="C24" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Puli</v>
+        <v>Malom</v>
       </c>
       <c r="D24" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Vizsla</v>
+        <v>Csend</v>
       </c>
       <c r="E24" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Kuvasz</v>
+        <v>Kakas</v>
       </c>
       <c r="F24" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Pumi</v>
+        <v>Vihar</v>
       </c>
       <c r="G24" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1))</f>
@@ -8379,23 +8393,23 @@
       </c>
       <c r="B25" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Aminek nyelve van</v>
+        <v>Aminek lába van</v>
       </c>
       <c r="C25" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Cipő</v>
+        <v>Asztal</v>
       </c>
       <c r="D25" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Harang</v>
+        <v>Gomba</v>
       </c>
       <c r="E25" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Öv</v>
+        <v>Nadrág</v>
       </c>
       <c r="F25" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Mérleg</v>
+        <v>Szék</v>
       </c>
       <c r="G25" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1))</f>
@@ -8408,27 +8422,27 @@
       </c>
       <c r="B26" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Egy betű cseréjével vármegye</v>
+        <v>Palindrom szavak</v>
       </c>
       <c r="C26" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Fehér</v>
+        <v>Görög</v>
       </c>
       <c r="D26" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Bélés</v>
+        <v>Indián</v>
       </c>
       <c r="E26" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Rest</v>
+        <v>Kerek</v>
       </c>
       <c r="F26" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Volna</v>
+        <v>Pap</v>
       </c>
       <c r="G26" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1))</f>
-        <v>Fejér, Békés, Pest, Tolna</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix live puzzle rsz-012: Kő -> Csap in TŰZ + ___
"Tűzkő" swapped for "Tűzcsap" in today's (2026-10-04) level 2 group.
Same id and date; rebuilt with `build.py --javitas rsz-012`. Saved
in-progress games referencing "Kő" reset via the existing stale-state guard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feladvanyok.xlsx
+++ b/feladvanyok.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0a3b2d023d0b90a2/Dokumentumok/GitHub/rokonszavak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="11_4BC928A0A355CC1831E4553E7CBF07CDD619E1D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{628C337C-280F-4B15-A767-E1BC83D40D2F}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="11_4BC928A0A355CC1831E4553E7CBF07CDD619E1D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{885B2CDE-6310-4B00-964D-4E043AFEDFFA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Segéd" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="Játék" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="466">
   <si>
     <t>Rokonszavak – feladványbank és gyakorlólap</t>
   </si>
@@ -626,9 +626,6 @@
     <t>Vihar</t>
   </si>
   <si>
-    <t>Aminek lába van</t>
-  </si>
-  <si>
     <t>Asztal</t>
   </si>
   <si>
@@ -639,9 +636,6 @@
   </si>
   <si>
     <t>Szék</t>
-  </si>
-  <si>
-    <t>Palindrom szavak</t>
   </si>
   <si>
     <t>Görög</t>
@@ -1475,7 +1469,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1496,19 +1490,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
+        <fgColor theme="3" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1540,7 +1522,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1554,12 +1536,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1645,10 +1621,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2207,7 +2179,7 @@
         <v>64</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>66</v>
@@ -2883,20 +2855,20 @@
         <v>3</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="E32" s="5"/>
       <c r="F32" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="G32" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>203</v>
-      </c>
       <c r="H32" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="J32" s="5"/>
     </row>
@@ -2911,17 +2883,17 @@
         <v>4</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="E33" s="5"/>
       <c r="F33" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>141</v>
@@ -2930,1019 +2902,1021 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C34" s="5">
         <v>1</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E34" s="5"/>
       <c r="F34" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="H34" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="I34" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>211</v>
       </c>
       <c r="J34" s="5"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C35" s="5">
         <v>2</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="H35" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="I35" s="5" t="s">
         <v>214</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="J35" s="5"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C36" s="5">
         <v>3</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E36" s="5"/>
       <c r="F36" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="H36" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G36" s="5" t="s">
+      <c r="I36" s="5" t="s">
         <v>219</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>221</v>
       </c>
       <c r="J36" s="5"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C37" s="5">
         <v>4</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E37" s="5"/>
       <c r="F37" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H37" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="G37" s="5" t="s">
+      <c r="I37" s="5" t="s">
         <v>224</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>226</v>
       </c>
       <c r="J37" s="5"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C38" s="5">
         <v>1</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E38" s="5"/>
       <c r="F38" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="H38" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="G38" s="5" t="s">
+      <c r="I38" s="5" t="s">
         <v>231</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="I38" s="5" t="s">
-        <v>233</v>
       </c>
       <c r="J38" s="5"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C39" s="5">
         <v>2</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E39" s="5"/>
       <c r="F39" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="H39" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="G39" s="5" t="s">
+      <c r="I39" s="5" t="s">
         <v>236</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="I39" s="5" t="s">
-        <v>238</v>
       </c>
       <c r="J39" s="5"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C40" s="5">
         <v>3</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H40" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="G40" s="5" t="s">
+      <c r="I40" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>243</v>
       </c>
       <c r="J40" s="5"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C41" s="5">
         <v>4</v>
       </c>
       <c r="D41" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="F41" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="G41" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="H41" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="G41" s="5" t="s">
+      <c r="I41" s="5" t="s">
         <v>247</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="I41" s="5" t="s">
-        <v>249</v>
       </c>
       <c r="J41" s="5"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C42" s="5">
         <v>1</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E42" s="5"/>
       <c r="F42" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="G42" s="5" t="s">
+      <c r="I42" s="5" t="s">
         <v>254</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="I42" s="5" t="s">
-        <v>256</v>
       </c>
       <c r="J42" s="5"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C43" s="5">
         <v>2</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E43" s="5"/>
       <c r="F43" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G43" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Csap</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="I43" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="J43" s="5"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C44" s="5">
         <v>3</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="G44" s="5" t="s">
+      <c r="I44" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>266</v>
       </c>
       <c r="J44" s="5"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C45" s="5">
         <v>4</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="H45" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="G45" s="5" t="s">
+      <c r="I45" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="H45" s="5" t="s">
+      <c r="J45" s="5" t="s">
         <v>270</v>
-      </c>
-      <c r="I45" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C46" s="5">
         <v>1</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="H46" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="G46" s="5" t="s">
+      <c r="I46" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>279</v>
       </c>
       <c r="J46" s="5"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C47" s="5">
         <v>2</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="H47" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="5" t="s">
+      <c r="I47" s="5" t="s">
         <v>282</v>
-      </c>
-      <c r="H47" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="I47" s="5" t="s">
-        <v>284</v>
       </c>
       <c r="J47" s="5"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C48" s="5">
         <v>3</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="H48" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="G48" s="5" t="s">
+      <c r="I48" s="5" t="s">
         <v>287</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>289</v>
       </c>
       <c r="J48" s="5"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C49" s="5">
         <v>4</v>
       </c>
       <c r="D49" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="E49" s="5" t="s">
+      <c r="G49" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="H49" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="G49" s="5" t="s">
+      <c r="I49" s="5" t="s">
         <v>293</v>
-      </c>
-      <c r="H49" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="I49" s="5" t="s">
-        <v>295</v>
       </c>
       <c r="J49" s="5"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C50" s="5">
         <v>1</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="H50" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="G50" s="5" t="s">
+      <c r="I50" s="5" t="s">
         <v>300</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="I50" s="5" t="s">
-        <v>302</v>
       </c>
       <c r="J50" s="5"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C51" s="5">
         <v>2</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="H51" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="G51" s="5" t="s">
+      <c r="I51" s="5" t="s">
         <v>305</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="I51" s="5" t="s">
-        <v>307</v>
       </c>
       <c r="J51" s="5"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C52" s="5">
         <v>3</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E52" s="5"/>
       <c r="F52" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="H52" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="G52" s="5" t="s">
+      <c r="I52" s="5" t="s">
         <v>310</v>
-      </c>
-      <c r="H52" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="I52" s="5" t="s">
-        <v>312</v>
       </c>
       <c r="J52" s="5"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C53" s="5">
         <v>4</v>
       </c>
       <c r="D53" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="F53" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="E53" s="5" t="s">
+      <c r="G53" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="F53" s="5" t="s">
+      <c r="H53" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="G53" s="5" t="s">
+      <c r="I53" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="H53" s="5" t="s">
+      <c r="J53" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="I53" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="J53" s="5" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C54" s="5">
         <v>1</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E54" s="5"/>
       <c r="F54" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="H54" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="G54" s="5" t="s">
+      <c r="I54" s="5" t="s">
         <v>324</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="I54" s="5" t="s">
-        <v>326</v>
       </c>
       <c r="J54" s="5"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C55" s="5">
         <v>2</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E55" s="5"/>
       <c r="F55" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="H55" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="G55" s="5" t="s">
+      <c r="I55" s="5" t="s">
         <v>329</v>
-      </c>
-      <c r="H55" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="I55" s="5" t="s">
-        <v>331</v>
       </c>
       <c r="J55" s="5"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C56" s="5">
         <v>3</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="E56" s="5"/>
       <c r="F56" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="H56" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="G56" s="5" t="s">
+      <c r="I56" s="5" t="s">
         <v>334</v>
-      </c>
-      <c r="H56" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="I56" s="5" t="s">
-        <v>336</v>
       </c>
       <c r="J56" s="5"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C57" s="5">
         <v>4</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="H57" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="G57" s="5" t="s">
+      <c r="I57" s="5" t="s">
         <v>339</v>
-      </c>
-      <c r="H57" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="I57" s="5" t="s">
-        <v>341</v>
       </c>
       <c r="J57" s="5"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C58" s="5">
         <v>1</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="H58" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="G58" s="5" t="s">
+      <c r="I58" s="5" t="s">
         <v>346</v>
-      </c>
-      <c r="H58" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="I58" s="5" t="s">
-        <v>348</v>
       </c>
       <c r="J58" s="5"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C59" s="5">
         <v>2</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="H59" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="G59" s="5" t="s">
+      <c r="I59" s="5" t="s">
         <v>351</v>
-      </c>
-      <c r="H59" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="I59" s="5" t="s">
-        <v>353</v>
       </c>
       <c r="J59" s="5"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C60" s="5">
         <v>3</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="H60" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="G60" s="5" t="s">
+      <c r="I60" s="5" t="s">
         <v>356</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="I60" s="5" t="s">
-        <v>358</v>
       </c>
       <c r="J60" s="5"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C61" s="5">
         <v>4</v>
       </c>
       <c r="D61" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="F61" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="G61" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="H61" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="G61" s="5" t="s">
+      <c r="I61" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="H61" s="5" t="s">
+      <c r="J61" s="5" t="s">
         <v>363</v>
-      </c>
-      <c r="I61" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="J61" s="5" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C62" s="5">
         <v>1</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="H62" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="G62" s="5" t="s">
+      <c r="I62" s="5" t="s">
         <v>370</v>
-      </c>
-      <c r="H62" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="I62" s="5" t="s">
-        <v>372</v>
       </c>
       <c r="J62" s="5"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C63" s="5">
         <v>2</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="G63" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="H63" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="G63" s="5" t="s">
+      <c r="I63" s="5" t="s">
         <v>375</v>
-      </c>
-      <c r="H63" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="I63" s="5" t="s">
-        <v>377</v>
       </c>
       <c r="J63" s="5"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C64" s="5">
         <v>3</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="G64" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="H64" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="G64" s="5" t="s">
+      <c r="I64" s="5" t="s">
         <v>380</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>382</v>
       </c>
       <c r="J64" s="5"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C65" s="5">
         <v>4</v>
       </c>
       <c r="D65" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="F65" s="5" t="s">
         <v>383</v>
       </c>
-      <c r="E65" s="5" t="s">
+      <c r="G65" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="F65" s="5" t="s">
+      <c r="H65" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="G65" s="5" t="s">
+      <c r="I65" s="5" t="s">
         <v>386</v>
-      </c>
-      <c r="H65" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="I65" s="5" t="s">
-        <v>388</v>
       </c>
       <c r="J65" s="5"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C66" s="5">
         <v>1</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="H66" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="G66" s="5" t="s">
+      <c r="I66" s="5" t="s">
         <v>393</v>
-      </c>
-      <c r="H66" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="I66" s="5" t="s">
-        <v>395</v>
       </c>
       <c r="J66" s="5"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C67" s="5">
         <v>2</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="G67" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="H67" s="5" t="s">
+        <v>396</v>
+      </c>
+      <c r="I67" s="5" t="s">
         <v>397</v>
-      </c>
-      <c r="H67" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="I67" s="5" t="s">
-        <v>399</v>
       </c>
       <c r="J67" s="5"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C68" s="5">
         <v>3</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="H68" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="G68" s="5" t="s">
+      <c r="I68" s="5" t="s">
         <v>402</v>
-      </c>
-      <c r="H68" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="I68" s="5" t="s">
-        <v>404</v>
       </c>
       <c r="J68" s="5"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C69" s="5">
         <v>4</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H69" s="5" t="s">
         <v>35</v>
@@ -3954,230 +3928,230 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C70" s="5">
         <v>1</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="H70" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="G70" s="5" t="s">
+      <c r="I70" s="5" t="s">
         <v>412</v>
-      </c>
-      <c r="H70" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="I70" s="5" t="s">
-        <v>414</v>
       </c>
       <c r="J70" s="5"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C71" s="5">
         <v>2</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E71" s="5"/>
       <c r="F71" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="H71" s="5" t="s">
         <v>416</v>
       </c>
-      <c r="G71" s="5" t="s">
+      <c r="I71" s="5" t="s">
         <v>417</v>
-      </c>
-      <c r="H71" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="I71" s="5" t="s">
-        <v>419</v>
       </c>
       <c r="J71" s="5"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C72" s="5">
         <v>3</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E72" s="5"/>
       <c r="F72" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="H72" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="G72" s="5" t="s">
+      <c r="I72" s="5" t="s">
         <v>422</v>
-      </c>
-      <c r="H72" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="I72" s="5" t="s">
-        <v>424</v>
       </c>
       <c r="J72" s="5"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C73" s="5">
         <v>4</v>
       </c>
       <c r="D73" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="F73" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="E73" s="5" t="s">
+      <c r="G73" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="H73" s="5" t="s">
         <v>427</v>
       </c>
-      <c r="G73" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="H73" s="5" t="s">
-        <v>429</v>
-      </c>
       <c r="I73" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J73" s="5"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C74" s="5">
         <v>1</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E74" s="5"/>
       <c r="F74" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="H74" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="G74" s="5" t="s">
+      <c r="I74" s="5" t="s">
         <v>434</v>
-      </c>
-      <c r="H74" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="I74" s="5" t="s">
-        <v>436</v>
       </c>
       <c r="J74" s="5"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C75" s="5">
         <v>2</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="E75" s="5"/>
       <c r="F75" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="H75" s="5" t="s">
         <v>438</v>
       </c>
-      <c r="G75" s="5" t="s">
+      <c r="I75" s="5" t="s">
         <v>439</v>
-      </c>
-      <c r="H75" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="I75" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="J75" s="5"/>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C76" s="5">
         <v>3</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E76" s="5"/>
       <c r="F76" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="H76" s="5" t="s">
         <v>443</v>
       </c>
-      <c r="G76" s="5" t="s">
+      <c r="I76" s="5" t="s">
         <v>444</v>
-      </c>
-      <c r="H76" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="I76" s="5" t="s">
-        <v>446</v>
       </c>
       <c r="J76" s="5"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C77" s="5">
         <v>4</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="E77" s="5"/>
       <c r="F77" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="H77" s="5" t="s">
         <v>448</v>
       </c>
-      <c r="G77" s="5" t="s">
+      <c r="I77" s="5" t="s">
         <v>449</v>
       </c>
-      <c r="H77" s="5" t="s">
+      <c r="J77" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="I77" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="J77" s="5" t="s">
-        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -4196,14 +4170,14 @@
         <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -4338,7 +4312,7 @@
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -4353,7 +4327,7 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -4368,7 +4342,7 @@
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -4383,7 +4357,7 @@
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -4398,7 +4372,7 @@
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -4413,7 +4387,7 @@
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -4428,7 +4402,7 @@
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -4443,7 +4417,7 @@
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -4458,7 +4432,7 @@
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -4473,7 +4447,7 @@
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -4488,7 +4462,7 @@
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -5708,7 +5682,7 @@
         <v>1</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
@@ -5721,7 +5695,7 @@
         <v>2</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D115" s="2"/>
       <c r="E115" s="2"/>
@@ -5760,7 +5734,7 @@
         <v>5</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
@@ -5773,7 +5747,7 @@
         <v>6</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
@@ -5812,7 +5786,7 @@
         <v>9</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D122" s="2"/>
       <c r="E122" s="2"/>
@@ -5838,7 +5812,7 @@
         <v>11</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D124" s="2"/>
       <c r="E124" s="2"/>
@@ -5890,7 +5864,7 @@
         <v>15</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D128" s="2"/>
       <c r="E128" s="2"/>
@@ -5903,1691 +5877,1691 @@
         <v>16</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B130" s="2">
         <v>1</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B131" s="2">
         <v>2</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B132" s="2">
         <v>3</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B133" s="2">
         <v>4</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D133" s="2"/>
       <c r="E133" s="2"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B134" s="2">
         <v>5</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D134" s="2"/>
       <c r="E134" s="2"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B135" s="2">
         <v>6</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D135" s="2"/>
       <c r="E135" s="2"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B136" s="2">
         <v>7</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D136" s="2"/>
       <c r="E136" s="2"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B137" s="2">
         <v>8</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D137" s="2"/>
       <c r="E137" s="2"/>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B138" s="2">
         <v>9</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D138" s="2"/>
       <c r="E138" s="2"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B139" s="2">
         <v>10</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D139" s="2"/>
       <c r="E139" s="2"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B140" s="2">
         <v>11</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D140" s="2"/>
       <c r="E140" s="2"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B141" s="2">
         <v>12</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D141" s="2"/>
       <c r="E141" s="2"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B142" s="2">
         <v>13</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D142" s="2"/>
       <c r="E142" s="2"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B143" s="2">
         <v>14</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D143" s="2"/>
       <c r="E143" s="2"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B144" s="2">
         <v>15</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D144" s="2"/>
       <c r="E144" s="2"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B145" s="2">
         <v>16</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D145" s="2"/>
       <c r="E145" s="2"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B146" s="2">
         <v>1</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D146" s="2"/>
       <c r="E146" s="2"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B147" s="2">
         <v>2</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D147" s="2"/>
       <c r="E147" s="2"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B148" s="2">
         <v>3</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D148" s="2"/>
       <c r="E148" s="2"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B149" s="2">
         <v>4</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D149" s="2"/>
       <c r="E149" s="2"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B150" s="2">
         <v>5</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B151" s="2">
         <v>6</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B152" s="2">
         <v>7</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B153" s="2">
         <v>8</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D153" s="2"/>
       <c r="E153" s="2"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B154" s="2">
         <v>9</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D154" s="2"/>
       <c r="E154" s="2"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B155" s="2">
         <v>10</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B156" s="2">
         <v>11</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B157" s="2">
         <v>12</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B158" s="2">
         <v>13</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B159" s="2">
         <v>14</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D159" s="2"/>
       <c r="E159" s="2"/>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B160" s="2">
         <v>15</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D160" s="2"/>
       <c r="E160" s="2"/>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B161" s="2">
         <v>16</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D161" s="2"/>
       <c r="E161" s="2"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B162" s="2">
         <v>1</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B163" s="2">
         <v>2</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D163" s="2"/>
       <c r="E163" s="2"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B164" s="2">
         <v>3</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D164" s="2"/>
       <c r="E164" s="2"/>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B165" s="2">
         <v>4</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D165" s="2"/>
       <c r="E165" s="2"/>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B166" s="2">
         <v>5</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B167" s="2">
         <v>6</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D167" s="2"/>
       <c r="E167" s="2"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B168" s="2">
         <v>7</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B169" s="2">
         <v>8</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B170" s="2">
         <v>9</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B171" s="2">
         <v>10</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D171" s="2"/>
       <c r="E171" s="2"/>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B172" s="2">
         <v>11</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D172" s="2"/>
       <c r="E172" s="2"/>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B173" s="2">
         <v>12</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B174" s="2">
         <v>13</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D174" s="2"/>
       <c r="E174" s="2"/>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B175" s="2">
         <v>14</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D175" s="2"/>
       <c r="E175" s="2"/>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B176" s="2">
         <v>15</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D176" s="2"/>
       <c r="E176" s="2"/>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B177" s="2">
         <v>16</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D177" s="2"/>
       <c r="E177" s="2"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B178" s="2">
         <v>1</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D178" s="2"/>
       <c r="E178" s="2"/>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B179" s="2">
         <v>2</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D179" s="2"/>
       <c r="E179" s="2"/>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B180" s="2">
         <v>3</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D180" s="2"/>
       <c r="E180" s="2"/>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B181" s="2">
         <v>4</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D181" s="2"/>
       <c r="E181" s="2"/>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B182" s="2">
         <v>5</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D182" s="2"/>
       <c r="E182" s="2"/>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B183" s="2">
         <v>6</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D183" s="2"/>
       <c r="E183" s="2"/>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B184" s="2">
         <v>7</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D184" s="2"/>
       <c r="E184" s="2"/>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B185" s="2">
         <v>8</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D185" s="2"/>
       <c r="E185" s="2"/>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B186" s="2">
         <v>9</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D186" s="2"/>
       <c r="E186" s="2"/>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B187" s="2">
         <v>10</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D187" s="2"/>
       <c r="E187" s="2"/>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B188" s="2">
         <v>11</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D188" s="2"/>
       <c r="E188" s="2"/>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B189" s="2">
         <v>12</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D189" s="2"/>
       <c r="E189" s="2"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B190" s="2">
         <v>13</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D190" s="2"/>
       <c r="E190" s="2"/>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B191" s="2">
         <v>14</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D191" s="2"/>
       <c r="E191" s="2"/>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B192" s="2">
         <v>15</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D192" s="2"/>
       <c r="E192" s="2"/>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B193" s="2">
         <v>16</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D193" s="2"/>
       <c r="E193" s="2"/>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B194" s="2">
         <v>1</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D194" s="2"/>
       <c r="E194" s="2"/>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B195" s="2">
         <v>2</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D195" s="2"/>
       <c r="E195" s="2"/>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B196" s="2">
         <v>3</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D196" s="2"/>
       <c r="E196" s="2"/>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B197" s="2">
         <v>4</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D197" s="2"/>
       <c r="E197" s="2"/>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B198" s="2">
         <v>5</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D198" s="2"/>
       <c r="E198" s="2"/>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B199" s="2">
         <v>6</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D199" s="2"/>
       <c r="E199" s="2"/>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B200" s="2">
         <v>7</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="D200" s="2"/>
       <c r="E200" s="2"/>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B201" s="2">
         <v>8</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D201" s="2"/>
       <c r="E201" s="2"/>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B202" s="2">
         <v>9</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D202" s="2"/>
       <c r="E202" s="2"/>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B203" s="2">
         <v>10</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D203" s="2"/>
       <c r="E203" s="2"/>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B204" s="2">
         <v>11</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D204" s="2"/>
       <c r="E204" s="2"/>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B205" s="2">
         <v>12</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D205" s="2"/>
       <c r="E205" s="2"/>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B206" s="2">
         <v>13</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="D206" s="2"/>
       <c r="E206" s="2"/>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B207" s="2">
         <v>14</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D207" s="2"/>
       <c r="E207" s="2"/>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B208" s="2">
         <v>15</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D208" s="2"/>
       <c r="E208" s="2"/>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B209" s="2">
         <v>16</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D209" s="2"/>
       <c r="E209" s="2"/>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B210" s="2">
         <v>1</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D210" s="2"/>
       <c r="E210" s="2"/>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B211" s="2">
         <v>2</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D211" s="2"/>
       <c r="E211" s="2"/>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B212" s="2">
         <v>3</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D212" s="2"/>
       <c r="E212" s="2"/>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B213" s="2">
         <v>4</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D213" s="2"/>
       <c r="E213" s="2"/>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B214" s="2">
         <v>5</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D214" s="2"/>
       <c r="E214" s="2"/>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B215" s="2">
         <v>6</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D215" s="2"/>
       <c r="E215" s="2"/>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B216" s="2">
         <v>7</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="D216" s="2"/>
       <c r="E216" s="2"/>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B217" s="2">
         <v>8</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D217" s="2"/>
       <c r="E217" s="2"/>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B218" s="2">
         <v>9</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D218" s="2"/>
       <c r="E218" s="2"/>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B219" s="2">
         <v>10</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D219" s="2"/>
       <c r="E219" s="2"/>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B220" s="2">
         <v>11</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D220" s="2"/>
       <c r="E220" s="2"/>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B221" s="2">
         <v>12</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D221" s="2"/>
       <c r="E221" s="2"/>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B222" s="2">
         <v>13</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D222" s="2"/>
       <c r="E222" s="2"/>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B223" s="2">
         <v>14</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="D223" s="2"/>
       <c r="E223" s="2"/>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B224" s="2">
         <v>15</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D224" s="2"/>
       <c r="E224" s="2"/>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B225" s="2">
         <v>16</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D225" s="2"/>
       <c r="E225" s="2"/>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B226" s="2">
         <v>1</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D226" s="2"/>
       <c r="E226" s="2"/>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B227" s="2">
         <v>2</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D227" s="2"/>
       <c r="E227" s="2"/>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B228" s="2">
         <v>3</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="D228" s="2"/>
       <c r="E228" s="2"/>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B229" s="2">
         <v>4</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D229" s="2"/>
       <c r="E229" s="2"/>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B230" s="2">
         <v>5</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D230" s="2"/>
       <c r="E230" s="2"/>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B231" s="2">
         <v>6</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D231" s="2"/>
       <c r="E231" s="2"/>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B232" s="2">
         <v>7</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D232" s="2"/>
       <c r="E232" s="2"/>
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A233" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B233" s="2">
         <v>8</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="D233" s="2"/>
       <c r="E233" s="2"/>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A234" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B234" s="2">
         <v>9</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D234" s="2"/>
       <c r="E234" s="2"/>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A235" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B235" s="2">
         <v>10</v>
       </c>
       <c r="C235" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D235" s="2"/>
       <c r="E235" s="2"/>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A236" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B236" s="2">
         <v>11</v>
       </c>
       <c r="C236" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D236" s="2"/>
       <c r="E236" s="2"/>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A237" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B237" s="2">
         <v>12</v>
       </c>
       <c r="C237" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D237" s="2"/>
       <c r="E237" s="2"/>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A238" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B238" s="2">
         <v>13</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="D238" s="2"/>
       <c r="E238" s="2"/>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A239" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B239" s="2">
         <v>14</v>
       </c>
       <c r="C239" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D239" s="2"/>
       <c r="E239" s="2"/>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A240" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B240" s="2">
         <v>15</v>
       </c>
       <c r="C240" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D240" s="2"/>
       <c r="E240" s="2"/>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A241" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B241" s="2">
         <v>16</v>
       </c>
       <c r="C241" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D241" s="2"/>
       <c r="E241" s="2"/>
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A242" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B242" s="2">
         <v>1</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D242" s="2"/>
       <c r="E242" s="2"/>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A243" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B243" s="2">
         <v>2</v>
       </c>
       <c r="C243" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D243" s="2"/>
       <c r="E243" s="2"/>
     </row>
     <row r="244" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A244" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B244" s="2">
         <v>3</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D244" s="2"/>
       <c r="E244" s="2"/>
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A245" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B245" s="2">
         <v>4</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D245" s="2"/>
       <c r="E245" s="2"/>
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A246" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B246" s="2">
         <v>5</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D246" s="2"/>
       <c r="E246" s="2"/>
     </row>
     <row r="247" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A247" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B247" s="2">
         <v>6</v>
       </c>
       <c r="C247" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D247" s="2"/>
       <c r="E247" s="2"/>
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A248" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B248" s="2">
         <v>7</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D248" s="2"/>
       <c r="E248" s="2"/>
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A249" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B249" s="2">
         <v>8</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D249" s="2"/>
       <c r="E249" s="2"/>
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A250" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B250" s="2">
         <v>9</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D250" s="2"/>
       <c r="E250" s="2"/>
     </row>
     <row r="251" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A251" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B251" s="2">
         <v>10</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D251" s="2"/>
       <c r="E251" s="2"/>
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A252" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B252" s="2">
         <v>11</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D252" s="2"/>
       <c r="E252" s="2"/>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A253" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B253" s="2">
         <v>12</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D253" s="2"/>
       <c r="E253" s="2"/>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A254" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B254" s="2">
         <v>13</v>
       </c>
       <c r="C254" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D254" s="2"/>
       <c r="E254" s="2"/>
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A255" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B255" s="2">
         <v>14</v>
       </c>
       <c r="C255" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D255" s="2"/>
       <c r="E255" s="2"/>
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A256" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B256" s="2">
         <v>15</v>
       </c>
       <c r="C256" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D256" s="2"/>
       <c r="E256" s="2"/>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A257" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B257" s="2">
         <v>16</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D257" s="2"/>
       <c r="E257" s="2"/>
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A258" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B258" s="2">
         <v>1</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D258" s="2"/>
       <c r="E258" s="2"/>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A259" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B259" s="2">
         <v>2</v>
@@ -7600,124 +7574,124 @@
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A260" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B260" s="2">
         <v>3</v>
       </c>
       <c r="C260" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D260" s="2"/>
       <c r="E260" s="2"/>
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A261" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B261" s="2">
         <v>4</v>
       </c>
       <c r="C261" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D261" s="2"/>
       <c r="E261" s="2"/>
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A262" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B262" s="2">
         <v>5</v>
       </c>
       <c r="C262" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D262" s="2"/>
       <c r="E262" s="2"/>
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A263" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B263" s="2">
         <v>6</v>
       </c>
       <c r="C263" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="D263" s="2"/>
       <c r="E263" s="2"/>
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A264" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B264" s="2">
         <v>7</v>
       </c>
       <c r="C264" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D264" s="2"/>
       <c r="E264" s="2"/>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A265" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B265" s="2">
         <v>8</v>
       </c>
       <c r="C265" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D265" s="2"/>
       <c r="E265" s="2"/>
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A266" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B266" s="2">
         <v>9</v>
       </c>
       <c r="C266" s="2" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D266" s="2"/>
       <c r="E266" s="2"/>
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A267" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B267" s="2">
         <v>10</v>
       </c>
       <c r="C267" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="D267" s="2"/>
       <c r="E267" s="2"/>
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A268" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B268" s="2">
         <v>11</v>
       </c>
       <c r="C268" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D268" s="2"/>
       <c r="E268" s="2"/>
     </row>
     <row r="269" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A269" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B269" s="2">
         <v>12</v>
@@ -7730,468 +7704,468 @@
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A270" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B270" s="2">
         <v>13</v>
       </c>
       <c r="C270" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D270" s="2"/>
       <c r="E270" s="2"/>
     </row>
     <row r="271" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A271" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B271" s="2">
         <v>14</v>
       </c>
       <c r="C271" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D271" s="2"/>
       <c r="E271" s="2"/>
     </row>
     <row r="272" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A272" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B272" s="2">
         <v>15</v>
       </c>
       <c r="C272" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="D272" s="2"/>
       <c r="E272" s="2"/>
     </row>
     <row r="273" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A273" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B273" s="2">
         <v>16</v>
       </c>
       <c r="C273" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D273" s="2"/>
       <c r="E273" s="2"/>
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A274" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B274" s="2">
         <v>1</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D274" s="2"/>
       <c r="E274" s="2"/>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A275" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B275" s="2">
         <v>2</v>
       </c>
       <c r="C275" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="D275" s="2"/>
       <c r="E275" s="2"/>
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A276" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B276" s="2">
         <v>3</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D276" s="2"/>
       <c r="E276" s="2"/>
     </row>
     <row r="277" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A277" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B277" s="2">
         <v>4</v>
       </c>
       <c r="C277" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D277" s="2"/>
       <c r="E277" s="2"/>
     </row>
     <row r="278" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A278" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B278" s="2">
         <v>5</v>
       </c>
       <c r="C278" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D278" s="2"/>
       <c r="E278" s="2"/>
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A279" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B279" s="2">
         <v>6</v>
       </c>
       <c r="C279" s="2" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D279" s="2"/>
       <c r="E279" s="2"/>
     </row>
     <row r="280" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A280" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B280" s="2">
         <v>7</v>
       </c>
       <c r="C280" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D280" s="2"/>
       <c r="E280" s="2"/>
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A281" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B281" s="2">
         <v>8</v>
       </c>
       <c r="C281" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D281" s="2"/>
       <c r="E281" s="2"/>
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A282" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B282" s="2">
         <v>9</v>
       </c>
       <c r="C282" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D282" s="2"/>
       <c r="E282" s="2"/>
     </row>
     <row r="283" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A283" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B283" s="2">
         <v>10</v>
       </c>
       <c r="C283" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D283" s="2"/>
       <c r="E283" s="2"/>
     </row>
     <row r="284" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A284" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B284" s="2">
         <v>11</v>
       </c>
       <c r="C284" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D284" s="2"/>
       <c r="E284" s="2"/>
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A285" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B285" s="2">
         <v>12</v>
       </c>
       <c r="C285" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D285" s="2"/>
       <c r="E285" s="2"/>
     </row>
     <row r="286" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A286" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B286" s="2">
         <v>13</v>
       </c>
       <c r="C286" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D286" s="2"/>
       <c r="E286" s="2"/>
     </row>
     <row r="287" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A287" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B287" s="2">
         <v>14</v>
       </c>
       <c r="C287" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D287" s="2"/>
       <c r="E287" s="2"/>
     </row>
     <row r="288" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A288" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B288" s="2">
         <v>15</v>
       </c>
       <c r="C288" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D288" s="2"/>
       <c r="E288" s="2"/>
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A289" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B289" s="2">
         <v>16</v>
       </c>
       <c r="C289" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D289" s="2"/>
       <c r="E289" s="2"/>
     </row>
     <row r="290" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A290" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B290" s="2">
         <v>1</v>
       </c>
       <c r="C290" s="2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D290" s="2"/>
       <c r="E290" s="2"/>
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A291" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B291" s="2">
         <v>2</v>
       </c>
       <c r="C291" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D291" s="2"/>
       <c r="E291" s="2"/>
     </row>
     <row r="292" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A292" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B292" s="2">
         <v>3</v>
       </c>
       <c r="C292" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D292" s="2"/>
       <c r="E292" s="2"/>
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A293" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B293" s="2">
         <v>4</v>
       </c>
       <c r="C293" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D293" s="2"/>
       <c r="E293" s="2"/>
     </row>
     <row r="294" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A294" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B294" s="2">
         <v>5</v>
       </c>
       <c r="C294" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D294" s="2"/>
       <c r="E294" s="2"/>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A295" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B295" s="2">
         <v>6</v>
       </c>
       <c r="C295" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D295" s="2"/>
       <c r="E295" s="2"/>
     </row>
     <row r="296" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A296" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B296" s="2">
         <v>7</v>
       </c>
       <c r="C296" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D296" s="2"/>
       <c r="E296" s="2"/>
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A297" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B297" s="2">
         <v>8</v>
       </c>
       <c r="C297" s="2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D297" s="2"/>
       <c r="E297" s="2"/>
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A298" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B298" s="2">
         <v>9</v>
       </c>
       <c r="C298" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="D298" s="2"/>
       <c r="E298" s="2"/>
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A299" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B299" s="2">
         <v>10</v>
       </c>
       <c r="C299" s="2" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D299" s="2"/>
       <c r="E299" s="2"/>
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A300" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B300" s="2">
         <v>11</v>
       </c>
       <c r="C300" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D300" s="2"/>
       <c r="E300" s="2"/>
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A301" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B301" s="2">
         <v>12</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D301" s="2"/>
       <c r="E301" s="2"/>
     </row>
     <row r="302" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A302" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B302" s="2">
         <v>13</v>
       </c>
       <c r="C302" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D302" s="2"/>
       <c r="E302" s="2"/>
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A303" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B303" s="2">
         <v>14</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D303" s="2"/>
       <c r="E303" s="2"/>
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A304" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B304" s="2">
         <v>15</v>
       </c>
       <c r="C304" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="D304" s="2"/>
       <c r="E304" s="2"/>
     </row>
     <row r="305" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A305" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B305" s="2">
         <v>16</v>
       </c>
       <c r="C305" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D305" s="2"/>
       <c r="E305" s="2"/>
@@ -8215,118 +8189,118 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>183</v>
+        <v>248</v>
       </c>
       <c r="C2" t="str">
         <f>VLOOKUP(B2,Feladványok!A:B,2,FALSE)</f>
-        <v>2026-10-01</v>
+        <v>2026-10-04</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="str">
+      <c r="A6" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+1-1)</f>
-        <v>Indián</v>
+        <v>Fog</v>
       </c>
       <c r="B6" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+2-1)</f>
-        <v>Szék</v>
+        <v>Kő</v>
       </c>
       <c r="C6" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+3-1)</f>
-        <v>Kapor</v>
-      </c>
-      <c r="D6" s="8" t="str">
+        <v>Csuka</v>
+      </c>
+      <c r="D6" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+4-1)</f>
-        <v>Csend</v>
+        <v>Ponty</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="str">
+      <c r="A7" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+5-1)</f>
-        <v>Görög</v>
+        <v>Keszeg</v>
       </c>
       <c r="B7" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+6-1)</f>
-        <v>Kerek</v>
-      </c>
-      <c r="C7" s="10" t="str">
+        <v>Veszély</v>
+      </c>
+      <c r="C7" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+7-1)</f>
-        <v>Bors</v>
-      </c>
-      <c r="D7" s="10" t="str">
+        <v>Fal</v>
+      </c>
+      <c r="D7" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+8-1)</f>
-        <v>Vihar</v>
+        <v>Vár</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="str">
+      <c r="A8" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+9-1)</f>
-        <v>Pap</v>
-      </c>
-      <c r="B8" s="9" t="str">
+        <v>Ég</v>
+      </c>
+      <c r="B8" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+10-1)</f>
-        <v>Kömény</v>
-      </c>
-      <c r="C8" s="8" t="str">
+        <v>Cipzár</v>
+      </c>
+      <c r="C8" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+11-1)</f>
-        <v>Gomba</v>
-      </c>
-      <c r="D8" s="9" t="str">
+        <v>Harcsa</v>
+      </c>
+      <c r="D8" s="8" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+12-1)</f>
-        <v>Kakas</v>
+        <v>Fésű</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+13-1)</f>
-        <v>Babér</v>
-      </c>
-      <c r="B9" s="9" t="str">
+        <v>Oltó</v>
+      </c>
+      <c r="B9" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+14-1)</f>
-        <v>Malom</v>
-      </c>
-      <c r="C9" s="9" t="str">
+        <v>Fűrész</v>
+      </c>
+      <c r="C9" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+15-1)</f>
-        <v>Asztal</v>
-      </c>
-      <c r="D9" s="10" t="str">
+        <v>Gereblye</v>
+      </c>
+      <c r="D9" s="7" t="str">
         <f>INDEX(Segéd!$C$2:$C$305,MATCH($B$2,Segéd!$A$2:$A$305,0)+16-1)</f>
-        <v>Nadrág</v>
+        <v>Nyúl</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -8335,23 +8309,23 @@
       </c>
       <c r="B23" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Fűszerek</v>
+        <v>Halak</v>
       </c>
       <c r="C23" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Kömény</v>
+        <v>Ponty</v>
       </c>
       <c r="D23" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Bors</v>
+        <v>Harcsa</v>
       </c>
       <c r="E23" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Kapor</v>
+        <v>Keszeg</v>
       </c>
       <c r="F23" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)</f>
-        <v>Babér</v>
+        <v>Csuka</v>
       </c>
       <c r="G23" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+1-1))</f>
@@ -8364,23 +8338,23 @@
       </c>
       <c r="B24" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>SZÉL + ___</v>
+        <v>TŰZ + ___</v>
       </c>
       <c r="C24" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Malom</v>
+        <v>Oltó</v>
       </c>
       <c r="D24" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Csend</v>
+        <v>Fal</v>
       </c>
       <c r="E24" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Kakas</v>
+        <v>Kő</v>
       </c>
       <c r="F24" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)</f>
-        <v>Vihar</v>
+        <v>Veszély</v>
       </c>
       <c r="G24" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+2-1))</f>
@@ -8393,23 +8367,23 @@
       </c>
       <c r="B25" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Aminek lába van</v>
+        <v>Aminek foga van</v>
       </c>
       <c r="C25" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Asztal</v>
+        <v>Fésű</v>
       </c>
       <c r="D25" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Gomba</v>
+        <v>Fűrész</v>
       </c>
       <c r="E25" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Nadrág</v>
+        <v>Gereblye</v>
       </c>
       <c r="F25" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)</f>
-        <v>Szék</v>
+        <v>Cipzár</v>
       </c>
       <c r="G25" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+3-1))</f>
@@ -8422,23 +8396,23 @@
       </c>
       <c r="B26" s="5" t="str">
         <f>INDEX(Feladványok!$D$2:$D$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Palindrom szavak</v>
+        <v>Főnév és ige is egyben</v>
       </c>
       <c r="C26" s="5" t="str">
         <f>INDEX(Feladványok!$F$2:$F$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Görög</v>
+        <v>Vár</v>
       </c>
       <c r="D26" s="5" t="str">
         <f>INDEX(Feladványok!$G$2:$G$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Indián</v>
+        <v>Fog</v>
       </c>
       <c r="E26" s="5" t="str">
         <f>INDEX(Feladványok!$H$2:$H$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Kerek</v>
+        <v>Nyúl</v>
       </c>
       <c r="F26" s="5" t="str">
         <f>INDEX(Feladványok!$I$2:$I$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)</f>
-        <v>Pap</v>
+        <v>Ég</v>
       </c>
       <c r="G26" s="5" t="str">
         <f>IF(INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1)="","",INDEX(Feladványok!$E$2:$E$77,MATCH($B$2,Feladványok!$A$2:$A$77,0)+4-1))</f>

</xml_diff>

<commit_message>
Fix live puzzle rsz-024: Malária -> Románc in "Ország rejtőzik a szóban"
Malária does not contain Mali. Románc hides Omán; note updated to
"Kína, Irán, India, Omán". Rebuilt with build.py --javitas rsz-024.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feladvanyok.xlsx
+++ b/feladvanyok.xlsx
@@ -1702,7 +1702,7 @@
     <t xml:space="preserve">Ország rejtőzik a szóban</t>
   </si>
   <si>
-    <t xml:space="preserve">Kína, Irán, India, Mali</t>
+    <t xml:space="preserve">Kína, Irán, India, Omán</t>
   </si>
   <si>
     <t xml:space="preserve">Kínál</t>
@@ -1714,7 +1714,7 @@
     <t xml:space="preserve">Indián</t>
   </si>
   <si>
-    <t xml:space="preserve">Malária</t>
+    <t xml:space="preserve">Románc</t>
   </si>
   <si>
     <t xml:space="preserve">rsz-001</t>

</xml_diff>